<commit_message>
Change Overdue And icon hide
</commit_message>
<xml_diff>
--- a/bin/Debug/Template/SparePartRequestSheetIPO.xlsx
+++ b/bin/Debug/Template/SparePartRequestSheetIPO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT-Project\MC-Dept-App\bin\Debug\Template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{990D04FE-AC4E-4A99-81B4-2649B36F474A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29D48CBE-18B0-434A-AAF4-DFCAD5B4AC36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BBFB412F-6E2A-4F5D-8DDF-BCB1C8845C69}"/>
   </bookViews>
@@ -230,7 +230,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -245,16 +245,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -276,6 +267,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="7" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -982,22 +983,22 @@
     <col min="7" max="7" width="10.140625" customWidth="1"/>
     <col min="8" max="8" width="15.85546875" customWidth="1"/>
     <col min="9" max="9" width="15.140625" customWidth="1"/>
-    <col min="10" max="10" width="18.85546875" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" style="16" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
+      <c r="I1" s="20"/>
+      <c r="J1" s="20"/>
     </row>
     <row r="2" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
@@ -1011,106 +1012,106 @@
       <c r="I2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="J2" s="6"/>
+      <c r="J2" s="17"/>
     </row>
     <row r="3" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="D3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="I3" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="9" t="s">
+      <c r="J3" s="14" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="11"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="7"/>
+      <c r="A4" s="7"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="10"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="15"/>
     </row>
     <row r="5" spans="1:10" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="21"/>
-      <c r="J5" s="20"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="21"/>
     </row>
     <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="17"/>
-      <c r="B7" s="17"/>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
+      <c r="A7" s="18"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
       <c r="G7" s="4"/>
       <c r="I7" s="4"/>
     </row>
     <row r="8" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17"/>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
+      <c r="A8" s="18"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
       <c r="G8" s="4"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
     </row>
     <row r="9" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="17"/>
-      <c r="B9" s="17"/>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
+      <c r="A9" s="18"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
       <c r="G9" s="3"/>
       <c r="I9" s="4"/>
     </row>
     <row r="10" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="11" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
     </row>
     <row r="12" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:10" ht="21.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>